<commit_message>
offline mode dengan psql
</commit_message>
<xml_diff>
--- a/static/TEMPLATE_IMPORT.xlsx
+++ b/static/TEMPLATE_IMPORT.xlsx
@@ -8,19 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NB329\IDLAPS CHECKPOINT\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C95A247-7AF7-4A95-A37F-36C714CFA323}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{844C298F-C1B0-414E-9702-9FFDC722BCD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="category" sheetId="2" r:id="rId1"/>
+    <sheet name="epc" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>epc</t>
   </si>
@@ -77,6 +83,12 @@
   </si>
   <si>
     <t>category_id</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>lap</t>
   </si>
 </sst>
 </file>
@@ -605,6 +617,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFECD702-9DCA-4B1F-9915-FB173D90B7BF}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>

</xml_diff>